<commit_message>
update numerical stage stepping
</commit_message>
<xml_diff>
--- a/assets/misc/Numerical_stage_stepping.xlsx
+++ b/assets/misc/Numerical_stage_stepping.xlsx
@@ -3,16 +3,16 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22430"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC862F60-8BDB-4D3B-A4E4-C91494CB79AE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D955ED4A-9006-4F6A-BC86-08BA0ACDF77E}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5760" yWindow="3432" windowWidth="17280" windowHeight="9072" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Numerical Stage Stepping" sheetId="6" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="alpha">'Numerical Stage Stepping'!$F$3</definedName>
-    <definedName name="X_bottom">'Numerical Stage Stepping'!$F$4</definedName>
+    <definedName name="alpha">'Numerical Stage Stepping'!$G$3</definedName>
+    <definedName name="X_bottom">'Numerical Stage Stepping'!$G$4</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -71,7 +71,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -107,6 +107,13 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="2" tint="-0.499984740745262"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -192,7 +199,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
@@ -205,6 +212,9 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Explanatory Text" xfId="2" builtinId="53"/>
@@ -347,73 +357,73 @@
                   <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.32203389830508478</c:v>
+                  <c:v>0.55555555555555558</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.32203389830508478</c:v>
+                  <c:v>0.55555555555555558</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.32203389830508478</c:v>
+                  <c:v>0.55555555555555558</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.47437582128777928</c:v>
+                  <c:v>0.86206896551724133</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.47437582128777928</c:v>
+                  <c:v>0.86206896551724133</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.47437582128777928</c:v>
+                  <c:v>0.86206896551724133</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.63164195598121375</c:v>
+                  <c:v>0.96899224806201545</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.63164195598121375</c:v>
+                  <c:v>0.96899224806201545</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.76514933566618326</c:v>
+                  <c:v>0.99364069952305245</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.76514933566618326</c:v>
+                  <c:v>0.99364069952305245</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.76514933566618326</c:v>
+                  <c:v>0.99364069952305245</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.86092272901593447</c:v>
+                  <c:v>0.99872163630552879</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.86092272901593447</c:v>
+                  <c:v>0.99872163630552879</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.86092272901593447</c:v>
+                  <c:v>0.99872163630552879</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.92163912304697015</c:v>
+                  <c:v>0.9997440655192269</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.92163912304697015</c:v>
+                  <c:v>0.9997440655192269</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.95716756559864158</c:v>
+                  <c:v>0.99994880262130581</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.95716756559864158</c:v>
+                  <c:v>0.99994880262130581</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.95716756559864158</c:v>
+                  <c:v>0.99994880262130581</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.97698975756255602</c:v>
+                  <c:v>0.99998976010485663</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.97698975756255602</c:v>
+                  <c:v>0.99998976010485663</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.97698975756255602</c:v>
+                  <c:v>0.99998976010485663</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.98775589032830391</c:v>
+                  <c:v>0.99999795200419428</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -428,76 +438,76 @@
                   <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.32203389830508478</c:v>
+                  <c:v>0.55555555555555558</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.32203389830508478</c:v>
+                  <c:v>0.55555555555555558</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.47437582128777928</c:v>
+                  <c:v>0.86206896551724133</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.47437582128777928</c:v>
+                  <c:v>0.86206896551724133</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.47437582128777928</c:v>
+                  <c:v>0.86206896551724133</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.63164195598121375</c:v>
+                  <c:v>0.96899224806201545</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.63164195598121375</c:v>
+                  <c:v>0.96899224806201545</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.63164195598121375</c:v>
+                  <c:v>0.96899224806201545</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.76514933566618326</c:v>
+                  <c:v>0.99364069952305245</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.76514933566618326</c:v>
+                  <c:v>0.99364069952305245</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.86092272901593447</c:v>
+                  <c:v>0.99872163630552879</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.86092272901593447</c:v>
+                  <c:v>0.99872163630552879</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.86092272901593447</c:v>
+                  <c:v>0.99872163630552879</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.92163912304697015</c:v>
+                  <c:v>0.9997440655192269</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.92163912304697015</c:v>
+                  <c:v>0.9997440655192269</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.92163912304697015</c:v>
+                  <c:v>0.9997440655192269</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.95716756559864158</c:v>
+                  <c:v>0.99994880262130581</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.95716756559864158</c:v>
+                  <c:v>0.99994880262130581</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.97698975756255602</c:v>
+                  <c:v>0.99998976010485663</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.97698975756255602</c:v>
+                  <c:v>0.99998976010485663</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.97698975756255602</c:v>
+                  <c:v>0.99998976010485663</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.98775589032830391</c:v>
+                  <c:v>0.99999795200419428</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.98775589032830391</c:v>
+                  <c:v>0.99999795200419428</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.98775589032830391</c:v>
+                  <c:v>0.99999795200419428</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -529,7 +539,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Numerical Stage Stepping'!$H$3:$H$23</c:f>
+              <c:f>'Numerical Stage Stepping'!$I$3:$I$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
@@ -601,7 +611,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'Numerical Stage Stepping'!$H$3:$H$23</c:f>
+              <c:f>'Numerical Stage Stepping'!$I$3:$I$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
@@ -700,78 +710,6 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'Numerical Stage Stepping'!$H$3:$H$23</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="21"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.05</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.1</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.15</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.2</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0.25</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0.3</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0.35</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0.4</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0.45</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0.5</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0.55000000000000004</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>0.6</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>0.65</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>0.7</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>0.75</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>0.8</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>0.85</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>0.9</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>0.95</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>1</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
               <c:f>'Numerical Stage Stepping'!$I$3:$I$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
@@ -780,61 +718,133 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>9.0909090909090912E-2</c:v>
+                  <c:v>0.05</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.17431192660550457</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.25110132158590304</c:v>
+                  <c:v>0.15</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.32203389830508478</c:v>
+                  <c:v>0.2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.38775510204081626</c:v>
+                  <c:v>0.25</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.44881889763779526</c:v>
+                  <c:v>0.3</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.50570342205323193</c:v>
+                  <c:v>0.35</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.55882352941176472</c:v>
+                  <c:v>0.4</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.60854092526690384</c:v>
+                  <c:v>0.45</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.65517241379310343</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.69899665551839452</c:v>
+                  <c:v>0.55000000000000004</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.74025974025974017</c:v>
+                  <c:v>0.6</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.77917981072555198</c:v>
+                  <c:v>0.65</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.81595092024539873</c:v>
+                  <c:v>0.7</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.85074626865671643</c:v>
+                  <c:v>0.75</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.88372093023255816</c:v>
+                  <c:v>0.8</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.91501416430594906</c:v>
+                  <c:v>0.85</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.94475138121546953</c:v>
+                  <c:v>0.9</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.97304582210242585</c:v>
+                  <c:v>0.95</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Numerical Stage Stepping'!$J$3:$J$23</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="21"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.20833333333333334</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.35714285714285715</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.46875</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.55555555555555558</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.625</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.68181818181818177</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.72916666666666674</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.76923076923076916</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.8035714285714286</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.83333333333333337</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.859375</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.88235294117647056</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.90277777777777779</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.92105263157894746</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.9375</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.95238095238095233</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.96590909090909083</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.97826086956521752</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.98958333333333337</c:v>
                 </c:pt>
                 <c:pt idx="20">
                   <c:v>1</c:v>
@@ -1629,13 +1639,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>1147280</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>34246</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
+      <xdr:col>24</xdr:col>
       <xdr:colOff>136988</xdr:colOff>
       <xdr:row>36</xdr:row>
       <xdr:rowOff>68494</xdr:rowOff>
@@ -1929,32 +1939,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6330743D-06A7-4F0B-B551-882A284364DF}">
-  <dimension ref="A1:FJ103"/>
+  <dimension ref="A1:FK103"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.5546875" customWidth="1"/>
     <col min="2" max="2" width="14.33203125" customWidth="1"/>
-    <col min="3" max="3" width="4.33203125" customWidth="1"/>
-    <col min="4" max="4" width="4.88671875" customWidth="1"/>
-    <col min="5" max="5" width="15.21875" customWidth="1"/>
-    <col min="7" max="7" width="5.77734375" customWidth="1"/>
-    <col min="10" max="10" width="17.109375" customWidth="1"/>
+    <col min="3" max="4" width="4.33203125" customWidth="1"/>
+    <col min="5" max="5" width="4.88671875" customWidth="1"/>
+    <col min="6" max="6" width="15.21875" customWidth="1"/>
+    <col min="8" max="8" width="5.77734375" customWidth="1"/>
+    <col min="11" max="11" width="17.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:166" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:167" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
         <v>6</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="11"/>
-      <c r="H1" s="8" t="s">
+      <c r="D1" s="12"/>
+      <c r="I1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="J1" s="9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>0</v>
       </c>
@@ -1964,15 +1975,16 @@
       <c r="C2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="D2" s="13"/>
+      <c r="I2" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="J2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="1"/>
-    </row>
-    <row r="3" spans="1:166" x14ac:dyDescent="0.3">
+      <c r="K2" s="1"/>
+    </row>
+    <row r="3" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A3">
         <f>X_bottom</f>
         <v>0.2</v>
@@ -1981,941 +1993,1264 @@
         <f>A3</f>
         <v>0.2</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="14"/>
+      <c r="D3" s="1"/>
+      <c r="F3" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="G3" s="6">
+        <v>5</v>
+      </c>
+      <c r="I3">
         <v>0</v>
       </c>
-      <c r="E3" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="F3" s="6">
-        <v>1.9</v>
-      </c>
-      <c r="H3">
+      <c r="J3">
+        <f t="shared" ref="J3:J23" si="0">(I3*alpha)/(1+I3*(alpha-1))</f>
         <v>0</v>
       </c>
-      <c r="I3">
-        <f>(H3*alpha)/(1+H3*(alpha-1))</f>
+      <c r="K3" s="3"/>
+      <c r="L3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="O3" s="2"/>
+      <c r="FK3">
         <v>0</v>
       </c>
-      <c r="J3" s="3"/>
-      <c r="K3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="N3" s="2"/>
-      <c r="FJ3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:166" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A4">
         <f>A3</f>
         <v>0.2</v>
       </c>
       <c r="B4">
         <f>A3*alpha/(1+A3*(alpha-1))</f>
-        <v>0.32203389830508478</v>
-      </c>
-      <c r="C4">
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="C4" s="14">
         <v>1</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="D4" s="1">
+        <f>25-C4</f>
+        <v>24</v>
+      </c>
+      <c r="F4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="6">
+      <c r="G4" s="6">
         <v>0.2</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>0.05</v>
       </c>
-      <c r="I4">
-        <f>(H4*alpha)/(1+H4*(alpha-1))</f>
-        <v>9.0909090909090912E-2</v>
-      </c>
-      <c r="J4" s="3"/>
-      <c r="N4" s="2"/>
-      <c r="FJ4">
+      <c r="J4">
+        <f t="shared" si="0"/>
+        <v>0.20833333333333334</v>
+      </c>
+      <c r="K4" s="3"/>
+      <c r="O4" s="2"/>
+      <c r="FK4">
         <v>1.0494752623688158E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A5">
         <f>B4</f>
-        <v>0.32203389830508478</v>
+        <v>0.55555555555555558</v>
       </c>
       <c r="B5">
         <f>A5</f>
-        <v>0.32203389830508478</v>
-      </c>
-      <c r="C5">
-        <v>2</v>
-      </c>
-      <c r="H5">
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="C5" s="14"/>
+      <c r="D5" s="1"/>
+      <c r="I5">
         <v>0.1</v>
       </c>
-      <c r="I5">
-        <f>(H5*alpha)/(1+H5*(alpha-1))</f>
-        <v>0.17431192660550457</v>
-      </c>
-      <c r="N5" s="2"/>
-      <c r="FJ5">
+      <c r="J5">
+        <f t="shared" si="0"/>
+        <v>0.35714285714285715</v>
+      </c>
+      <c r="O5" s="2"/>
+      <c r="FK5">
         <v>2.0979020979020983E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A6">
         <f>A5</f>
-        <v>0.32203389830508478</v>
+        <v>0.55555555555555558</v>
       </c>
       <c r="B6">
         <f>A6*alpha/(1+A6*(alpha-1))</f>
-        <v>0.47437582128777928</v>
-      </c>
-      <c r="C6">
-        <v>3</v>
-      </c>
-      <c r="H6">
+        <v>0.86206896551724133</v>
+      </c>
+      <c r="C6" s="14">
+        <v>2</v>
+      </c>
+      <c r="D6" s="1">
+        <f t="shared" ref="D6:D50" si="1">25-C6</f>
+        <v>23</v>
+      </c>
+      <c r="I6">
         <v>0.15</v>
       </c>
-      <c r="I6">
-        <f>(H6*alpha)/(1+H6*(alpha-1))</f>
-        <v>0.25110132158590304</v>
-      </c>
-      <c r="FJ6">
+      <c r="J6">
+        <f t="shared" si="0"/>
+        <v>0.46875</v>
+      </c>
+      <c r="FK6">
         <v>3.1452820768846729E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>A6</f>
-        <v>0.32203389830508478</v>
+        <v>0.55555555555555558</v>
       </c>
       <c r="B7">
         <f>A6*alpha/(1+A6*(alpha-1))</f>
-        <v>0.47437582128777928</v>
-      </c>
-      <c r="C7">
-        <v>4</v>
-      </c>
-      <c r="H7">
+        <v>0.86206896551724133</v>
+      </c>
+      <c r="C7" s="14"/>
+      <c r="D7" s="1"/>
+      <c r="I7">
         <v>0.2</v>
       </c>
-      <c r="I7">
-        <f>(H7*alpha)/(1+H7*(alpha-1))</f>
-        <v>0.32203389830508478</v>
-      </c>
-      <c r="FJ7">
+      <c r="J7">
+        <f t="shared" si="0"/>
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="FK7">
         <v>4.1916167664670663E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A8">
         <f>B7</f>
-        <v>0.47437582128777928</v>
+        <v>0.86206896551724133</v>
       </c>
       <c r="B8">
         <f>A8</f>
-        <v>0.47437582128777928</v>
-      </c>
-      <c r="C8">
-        <v>5</v>
-      </c>
-      <c r="H8">
+        <v>0.86206896551724133</v>
+      </c>
+      <c r="C8" s="14">
+        <v>3</v>
+      </c>
+      <c r="D8" s="1">
+        <f t="shared" si="1"/>
+        <v>22</v>
+      </c>
+      <c r="I8">
         <v>0.25</v>
       </c>
-      <c r="I8">
-        <f>(H8*alpha)/(1+H8*(alpha-1))</f>
-        <v>0.38775510204081626</v>
-      </c>
-      <c r="FJ8">
+      <c r="J8">
+        <f t="shared" si="0"/>
+        <v>0.625</v>
+      </c>
+      <c r="FK8">
         <v>5.2369077306733174E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A9">
         <f>A8</f>
-        <v>0.47437582128777928</v>
+        <v>0.86206896551724133</v>
       </c>
       <c r="B9">
         <f>A8*alpha/(1+A8*(alpha-1))</f>
-        <v>0.63164195598121375</v>
-      </c>
-      <c r="C9">
-        <v>6</v>
-      </c>
-      <c r="H9">
+        <v>0.96899224806201545</v>
+      </c>
+      <c r="C9" s="14"/>
+      <c r="D9" s="1"/>
+      <c r="I9">
         <v>0.3</v>
       </c>
-      <c r="I9">
-        <f>(H9*alpha)/(1+H9*(alpha-1))</f>
-        <v>0.44881889763779526</v>
-      </c>
-      <c r="FJ9">
+      <c r="J9">
+        <f t="shared" si="0"/>
+        <v>0.68181818181818177</v>
+      </c>
+      <c r="FK9">
         <v>6.2811565304087727E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A10">
-        <f t="shared" ref="A10" si="0">A9</f>
-        <v>0.47437582128777928</v>
+        <f t="shared" ref="A10" si="2">A9</f>
+        <v>0.86206896551724133</v>
       </c>
       <c r="B10">
         <f>A9*alpha/(1+A9*(alpha-1))</f>
-        <v>0.63164195598121375</v>
-      </c>
-      <c r="C10">
-        <v>7</v>
-      </c>
-      <c r="H10">
+        <v>0.96899224806201545</v>
+      </c>
+      <c r="C10" s="14">
+        <v>4</v>
+      </c>
+      <c r="D10" s="1">
+        <f t="shared" si="1"/>
+        <v>21</v>
+      </c>
+      <c r="I10">
         <v>0.35</v>
       </c>
-      <c r="I10">
-        <f>(H10*alpha)/(1+H10*(alpha-1))</f>
-        <v>0.50570342205323193</v>
-      </c>
-      <c r="FJ10">
+      <c r="J10">
+        <f t="shared" si="0"/>
+        <v>0.72916666666666674</v>
+      </c>
+      <c r="FK10">
         <v>7.3243647234678633E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A11">
-        <f t="shared" ref="A11:A27" si="1">B10</f>
-        <v>0.63164195598121375</v>
+        <f t="shared" ref="A11:A27" si="3">B10</f>
+        <v>0.96899224806201545</v>
       </c>
       <c r="B11">
-        <f t="shared" ref="B11" si="2">A11</f>
-        <v>0.63164195598121375</v>
-      </c>
-      <c r="C11">
-        <v>8</v>
-      </c>
-      <c r="H11">
+        <f t="shared" ref="B11" si="4">A11</f>
+        <v>0.96899224806201545</v>
+      </c>
+      <c r="C11" s="14"/>
+      <c r="D11" s="1"/>
+      <c r="I11">
         <v>0.4</v>
       </c>
-      <c r="I11">
-        <f>(H11*alpha)/(1+H11*(alpha-1))</f>
-        <v>0.55882352941176472</v>
-      </c>
-      <c r="FJ11">
+      <c r="J11">
+        <f t="shared" si="0"/>
+        <v>0.76923076923076916</v>
+      </c>
+      <c r="FK11">
         <v>8.3665338645418336E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A12">
-        <f t="shared" ref="A12" si="3">A11</f>
-        <v>0.63164195598121375</v>
+        <f t="shared" ref="A12" si="5">A11</f>
+        <v>0.96899224806201545</v>
       </c>
       <c r="B12">
         <f>A11*alpha/(1+A11*(alpha-1))</f>
-        <v>0.76514933566618326</v>
-      </c>
-      <c r="C12">
-        <v>9</v>
-      </c>
-      <c r="H12">
+        <v>0.99364069952305245</v>
+      </c>
+      <c r="C12" s="14">
+        <v>5</v>
+      </c>
+      <c r="D12" s="1">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+      <c r="I12">
         <v>0.45</v>
       </c>
-      <c r="I12">
-        <f>(H12*alpha)/(1+H12*(alpha-1))</f>
-        <v>0.60854092526690384</v>
-      </c>
-      <c r="FJ12">
+      <c r="J12">
+        <f t="shared" si="0"/>
+        <v>0.8035714285714286</v>
+      </c>
+      <c r="FK12">
         <v>9.4076655052264813E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A13">
-        <f t="shared" ref="A13" si="4">B12</f>
-        <v>0.76514933566618326</v>
+        <f t="shared" ref="A13" si="6">B12</f>
+        <v>0.99364069952305245</v>
       </c>
       <c r="B13">
-        <f t="shared" ref="B13" si="5">A13</f>
-        <v>0.76514933566618326</v>
-      </c>
-      <c r="C13">
-        <v>10</v>
-      </c>
-      <c r="H13">
+        <f t="shared" ref="B13" si="7">A13</f>
+        <v>0.99364069952305245</v>
+      </c>
+      <c r="C13" s="14"/>
+      <c r="D13" s="1"/>
+      <c r="I13">
         <v>0.5</v>
       </c>
-      <c r="I13">
-        <f>(H13*alpha)/(1+H13*(alpha-1))</f>
-        <v>0.65517241379310343</v>
-      </c>
-      <c r="FJ13">
+      <c r="J13">
+        <f t="shared" si="0"/>
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="FK13">
         <v>0.10447761194029853</v>
       </c>
     </row>
-    <row r="14" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A14">
-        <f t="shared" ref="A14:A15" si="6">A13</f>
-        <v>0.76514933566618326</v>
+        <f t="shared" ref="A14:A15" si="8">A13</f>
+        <v>0.99364069952305245</v>
       </c>
       <c r="B14">
         <f>A14*alpha/(1+A14*(alpha-1))</f>
-        <v>0.86092272901593447</v>
-      </c>
-      <c r="C14">
-        <v>11</v>
-      </c>
-      <c r="H14">
+        <v>0.99872163630552879</v>
+      </c>
+      <c r="C14" s="14">
+        <v>6</v>
+      </c>
+      <c r="D14" s="1">
+        <f t="shared" si="1"/>
+        <v>19</v>
+      </c>
+      <c r="E14" s="1"/>
+      <c r="I14">
         <v>0.55000000000000004</v>
       </c>
-      <c r="I14">
-        <f>(H14*alpha)/(1+H14*(alpha-1))</f>
-        <v>0.69899665551839452</v>
-      </c>
-      <c r="FJ14">
+      <c r="J14">
+        <f t="shared" si="0"/>
+        <v>0.859375</v>
+      </c>
+      <c r="FK14">
         <v>0.1148682247637991</v>
       </c>
     </row>
-    <row r="15" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A15">
-        <f t="shared" si="6"/>
-        <v>0.76514933566618326</v>
+        <f t="shared" si="8"/>
+        <v>0.99364069952305245</v>
       </c>
       <c r="B15">
         <f>A14*alpha/(1+A14*(alpha-1))</f>
-        <v>0.86092272901593447</v>
-      </c>
-      <c r="C15">
-        <v>12</v>
-      </c>
-      <c r="H15">
+        <v>0.99872163630552879</v>
+      </c>
+      <c r="C15" s="14"/>
+      <c r="D15" s="1"/>
+      <c r="I15">
         <v>0.6</v>
       </c>
-      <c r="I15">
-        <f>(H15*alpha)/(1+H15*(alpha-1))</f>
-        <v>0.74025974025974017</v>
-      </c>
-      <c r="FJ15">
+      <c r="J15">
+        <f t="shared" si="0"/>
+        <v>0.88235294117647056</v>
+      </c>
+      <c r="FK15">
         <v>0.12524850894632206</v>
       </c>
     </row>
-    <row r="16" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A16">
-        <f t="shared" ref="A16" si="7">B15</f>
-        <v>0.86092272901593447</v>
+        <f t="shared" ref="A16" si="9">B15</f>
+        <v>0.99872163630552879</v>
       </c>
       <c r="B16">
-        <f t="shared" ref="B16" si="8">A16</f>
-        <v>0.86092272901593447</v>
-      </c>
-      <c r="C16">
-        <v>13</v>
-      </c>
-      <c r="H16">
+        <f t="shared" ref="B16" si="10">A16</f>
+        <v>0.99872163630552879</v>
+      </c>
+      <c r="C16" s="14">
+        <v>7</v>
+      </c>
+      <c r="D16" s="1">
+        <f t="shared" si="1"/>
+        <v>18</v>
+      </c>
+      <c r="I16">
         <v>0.65</v>
       </c>
-      <c r="I16">
-        <f>(H16*alpha)/(1+H16*(alpha-1))</f>
-        <v>0.77917981072555198</v>
-      </c>
-      <c r="FJ16">
+      <c r="J16">
+        <f t="shared" si="0"/>
+        <v>0.90277777777777779</v>
+      </c>
+      <c r="FK16">
         <v>0.13561847988077497</v>
       </c>
     </row>
-    <row r="17" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A17">
-        <f t="shared" ref="A17:A18" si="9">A16</f>
-        <v>0.86092272901593447</v>
+        <f t="shared" ref="A17:A18" si="11">A16</f>
+        <v>0.99872163630552879</v>
       </c>
       <c r="B17">
         <f>A16*alpha/(1+A16*(alpha-1))</f>
-        <v>0.92163912304697015</v>
-      </c>
-      <c r="C17">
-        <v>14</v>
-      </c>
-      <c r="H17">
+        <v>0.9997440655192269</v>
+      </c>
+      <c r="C17" s="14"/>
+      <c r="D17" s="1"/>
+      <c r="I17">
         <v>0.7</v>
       </c>
-      <c r="I17">
-        <f>(H17*alpha)/(1+H17*(alpha-1))</f>
-        <v>0.81595092024539873</v>
-      </c>
-      <c r="FJ17">
+      <c r="J17">
+        <f t="shared" si="0"/>
+        <v>0.92105263157894746</v>
+      </c>
+      <c r="FK17">
         <v>0.14597815292949354</v>
       </c>
     </row>
-    <row r="18" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A18">
-        <f t="shared" si="9"/>
-        <v>0.86092272901593447</v>
+        <f t="shared" si="11"/>
+        <v>0.99872163630552879</v>
       </c>
       <c r="B18">
         <f>A17*alpha/(1+A17*(alpha-1))</f>
-        <v>0.92163912304697015</v>
-      </c>
-      <c r="C18">
-        <v>15</v>
-      </c>
-      <c r="H18">
+        <v>0.9997440655192269</v>
+      </c>
+      <c r="C18" s="14">
+        <v>8</v>
+      </c>
+      <c r="D18" s="1">
+        <f t="shared" si="1"/>
+        <v>17</v>
+      </c>
+      <c r="I18">
         <v>0.75</v>
       </c>
-      <c r="I18">
-        <f>(H18*alpha)/(1+H18*(alpha-1))</f>
-        <v>0.85074626865671643</v>
-      </c>
-      <c r="FJ18">
+      <c r="J18">
+        <f t="shared" si="0"/>
+        <v>0.9375</v>
+      </c>
+      <c r="FK18">
         <v>0.15632754342431762</v>
       </c>
     </row>
-    <row r="19" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A19">
-        <f t="shared" si="1"/>
-        <v>0.92163912304697015</v>
+        <f t="shared" si="3"/>
+        <v>0.9997440655192269</v>
       </c>
       <c r="B19">
-        <f t="shared" ref="B19:B27" si="10">A19</f>
-        <v>0.92163912304697015</v>
-      </c>
-      <c r="C19">
-        <v>16</v>
-      </c>
-      <c r="H19">
+        <f t="shared" ref="B19:B27" si="12">A19</f>
+        <v>0.9997440655192269</v>
+      </c>
+      <c r="C19" s="14"/>
+      <c r="D19" s="1"/>
+      <c r="I19">
         <v>0.8</v>
       </c>
-      <c r="I19">
-        <f>(H19*alpha)/(1+H19*(alpha-1))</f>
-        <v>0.88372093023255816</v>
-      </c>
-      <c r="FJ19">
+      <c r="J19">
+        <f t="shared" si="0"/>
+        <v>0.95238095238095233</v>
+      </c>
+      <c r="FK19">
         <v>0.16666666666666669</v>
       </c>
     </row>
-    <row r="20" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A20">
-        <f t="shared" ref="A20" si="11">A19</f>
-        <v>0.92163912304697015</v>
+        <f t="shared" ref="A20" si="13">A19</f>
+        <v>0.9997440655192269</v>
       </c>
       <c r="B20">
         <f>A19*alpha/(1+A19*(alpha-1))</f>
-        <v>0.95716756559864158</v>
-      </c>
-      <c r="C20">
-        <v>17</v>
-      </c>
-      <c r="H20">
+        <v>0.99994880262130581</v>
+      </c>
+      <c r="C20" s="14">
+        <v>9</v>
+      </c>
+      <c r="D20" s="1">
+        <f t="shared" si="1"/>
+        <v>16</v>
+      </c>
+      <c r="I20">
         <v>0.85</v>
       </c>
-      <c r="I20">
-        <f>(H20*alpha)/(1+H20*(alpha-1))</f>
-        <v>0.91501416430594906</v>
-      </c>
-      <c r="FJ20">
+      <c r="J20">
+        <f t="shared" si="0"/>
+        <v>0.96590909090909083</v>
+      </c>
+      <c r="FK20">
         <v>0.1769955379276153</v>
       </c>
     </row>
-    <row r="21" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A21">
-        <f t="shared" ref="A21" si="12">B20</f>
-        <v>0.95716756559864158</v>
+        <f t="shared" ref="A21" si="14">B20</f>
+        <v>0.99994880262130581</v>
       </c>
       <c r="B21">
-        <f t="shared" ref="B21" si="13">A21</f>
-        <v>0.95716756559864158</v>
-      </c>
-      <c r="C21">
-        <v>18</v>
-      </c>
-      <c r="H21">
+        <f t="shared" ref="B21" si="15">A21</f>
+        <v>0.99994880262130581</v>
+      </c>
+      <c r="C21" s="14"/>
+      <c r="D21" s="1"/>
+      <c r="I21">
         <v>0.9</v>
       </c>
-      <c r="I21">
-        <f>(H21*alpha)/(1+H21*(alpha-1))</f>
-        <v>0.94475138121546953</v>
-      </c>
-      <c r="FJ21">
+      <c r="J21">
+        <f t="shared" si="0"/>
+        <v>0.97826086956521752</v>
+      </c>
+      <c r="FK21">
         <v>0.1873141724479683</v>
       </c>
     </row>
-    <row r="22" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A22">
-        <f t="shared" ref="A22:A23" si="14">A21</f>
-        <v>0.95716756559864158</v>
+        <f t="shared" ref="A22:A23" si="16">A21</f>
+        <v>0.99994880262130581</v>
       </c>
       <c r="B22">
         <f>A22*alpha/(1+A22*(alpha-1))</f>
-        <v>0.97698975756255602</v>
-      </c>
-      <c r="C22">
-        <v>19</v>
-      </c>
-      <c r="H22">
+        <v>0.99998976010485663</v>
+      </c>
+      <c r="C22" s="14">
+        <v>10</v>
+      </c>
+      <c r="D22" s="1">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="I22">
         <v>0.95</v>
       </c>
-      <c r="I22">
-        <f>(H22*alpha)/(1+H22*(alpha-1))</f>
-        <v>0.97304582210242585</v>
-      </c>
-      <c r="FJ22">
+      <c r="J22">
+        <f t="shared" si="0"/>
+        <v>0.98958333333333337</v>
+      </c>
+      <c r="FK22">
         <v>0.1976225854383358</v>
       </c>
     </row>
-    <row r="23" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A23">
-        <f t="shared" si="14"/>
-        <v>0.95716756559864158</v>
+        <f t="shared" si="16"/>
+        <v>0.99994880262130581</v>
       </c>
       <c r="B23">
         <f>A22*alpha/(1+A22*(alpha-1))</f>
-        <v>0.97698975756255602</v>
-      </c>
-      <c r="C23">
-        <v>20</v>
-      </c>
-      <c r="H23">
+        <v>0.99998976010485663</v>
+      </c>
+      <c r="C23" s="14"/>
+      <c r="D23" s="1"/>
+      <c r="I23">
         <v>1</v>
       </c>
-      <c r="I23">
-        <f>(H23*alpha)/(1+H23*(alpha-1))</f>
+      <c r="J23">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="FJ23">
+      <c r="FK23">
         <v>0.20792079207920794</v>
       </c>
     </row>
-    <row r="24" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A24">
-        <f t="shared" ref="A24" si="15">B23</f>
-        <v>0.97698975756255602</v>
+        <f t="shared" ref="A24" si="17">B23</f>
+        <v>0.99998976010485663</v>
       </c>
       <c r="B24">
-        <f t="shared" ref="B24" si="16">A24</f>
-        <v>0.97698975756255602</v>
-      </c>
-      <c r="C24">
-        <v>21</v>
-      </c>
-      <c r="FJ24">
+        <f t="shared" ref="B24" si="18">A24</f>
+        <v>0.99998976010485663</v>
+      </c>
+      <c r="C24" s="14">
+        <v>11</v>
+      </c>
+      <c r="D24" s="1">
+        <f t="shared" si="1"/>
+        <v>14</v>
+      </c>
+      <c r="FK24">
         <v>0.2182088075210292</v>
       </c>
     </row>
-    <row r="25" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A25">
-        <f t="shared" ref="A25:A26" si="17">A24</f>
-        <v>0.97698975756255602</v>
+        <f t="shared" ref="A25:A26" si="19">A24</f>
+        <v>0.99998976010485663</v>
       </c>
       <c r="B25">
         <f>A24*alpha/(1+A24*(alpha-1))</f>
-        <v>0.98775589032830391</v>
-      </c>
-      <c r="C25">
-        <v>22</v>
-      </c>
-      <c r="FJ25">
+        <v>0.99999795200419428</v>
+      </c>
+      <c r="C25" s="14"/>
+      <c r="D25" s="1"/>
+      <c r="FK25">
         <v>0.22848664688427298</v>
       </c>
     </row>
-    <row r="26" spans="1:166" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:167" x14ac:dyDescent="0.3">
       <c r="A26">
-        <f t="shared" si="17"/>
-        <v>0.97698975756255602</v>
+        <f t="shared" si="19"/>
+        <v>0.99998976010485663</v>
       </c>
       <c r="B26">
         <f>A25*alpha/(1+A25*(alpha-1))</f>
-        <v>0.98775589032830391</v>
-      </c>
-      <c r="C26">
+        <v>0.99999795200419428</v>
+      </c>
+      <c r="C26" s="14">
+        <v>12</v>
+      </c>
+      <c r="D26" s="1">
+        <f t="shared" si="1"/>
+        <v>13</v>
+      </c>
+      <c r="FK26">
+        <v>0.23875432525951557</v>
+      </c>
+    </row>
+    <row r="27" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <f t="shared" si="3"/>
+        <v>0.99999795200419428</v>
+      </c>
+      <c r="B27">
+        <f t="shared" si="12"/>
+        <v>0.99999795200419428</v>
+      </c>
+      <c r="C27" s="14"/>
+      <c r="D27" s="1"/>
+      <c r="FK27">
+        <v>0.24901185770750989</v>
+      </c>
+    </row>
+    <row r="28" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <f>X_bottom</f>
+        <v>0.2</v>
+      </c>
+      <c r="B28">
+        <f>A28</f>
+        <v>0.2</v>
+      </c>
+      <c r="C28" s="14">
+        <v>13</v>
+      </c>
+      <c r="D28" s="1">
+        <f t="shared" si="1"/>
+        <v>12</v>
+      </c>
+      <c r="FK28">
+        <v>0.2592592592592593</v>
+      </c>
+    </row>
+    <row r="29" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <f>A28</f>
+        <v>0.2</v>
+      </c>
+      <c r="B29">
+        <f>A28*alpha/(1+A28*(alpha-1))</f>
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="C29" s="14"/>
+      <c r="D29" s="1"/>
+      <c r="FK29">
+        <v>0.26949654491609087</v>
+      </c>
+    </row>
+    <row r="30" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <f>B29</f>
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="B30">
+        <f>A30</f>
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="C30" s="14">
+        <v>14</v>
+      </c>
+      <c r="D30" s="1">
+        <f t="shared" si="1"/>
+        <v>11</v>
+      </c>
+      <c r="FK30">
+        <v>0.27972372964972869</v>
+      </c>
+    </row>
+    <row r="31" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <f>A30</f>
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="B31">
+        <f>A31*alpha/(1+A31*(alpha-1))</f>
+        <v>0.86206896551724133</v>
+      </c>
+      <c r="C31" s="14"/>
+      <c r="D31" s="1"/>
+      <c r="FK31">
+        <v>0.2899408284023669</v>
+      </c>
+    </row>
+    <row r="32" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <f>A31</f>
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="B32">
+        <f>A31*alpha/(1+A31*(alpha-1))</f>
+        <v>0.86206896551724133</v>
+      </c>
+      <c r="C32" s="14">
+        <v>15</v>
+      </c>
+      <c r="D32" s="1">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="FK32">
+        <v>0.30014785608674227</v>
+      </c>
+    </row>
+    <row r="33" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <f>B32</f>
+        <v>0.86206896551724133</v>
+      </c>
+      <c r="B33">
+        <f>A33</f>
+        <v>0.86206896551724133</v>
+      </c>
+      <c r="C33" s="14"/>
+      <c r="D33" s="1"/>
+      <c r="FK33">
+        <v>0.31034482758620685</v>
+      </c>
+    </row>
+    <row r="34" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <f>A33</f>
+        <v>0.86206896551724133</v>
+      </c>
+      <c r="B34">
+        <f>A33*alpha/(1+A33*(alpha-1))</f>
+        <v>0.96899224806201545</v>
+      </c>
+      <c r="C34" s="14">
+        <v>16</v>
+      </c>
+      <c r="D34" s="1">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="FK34">
+        <v>0.32053175775480058</v>
+      </c>
+    </row>
+    <row r="35" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <f t="shared" ref="A35" si="20">A34</f>
+        <v>0.86206896551724133</v>
+      </c>
+      <c r="B35">
+        <f>A34*alpha/(1+A34*(alpha-1))</f>
+        <v>0.96899224806201545</v>
+      </c>
+      <c r="C35" s="14"/>
+      <c r="D35" s="1"/>
+      <c r="FK35">
+        <v>0.33070866141732286</v>
+      </c>
+    </row>
+    <row r="36" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <f t="shared" ref="A36" si="21">B35</f>
+        <v>0.96899224806201545</v>
+      </c>
+      <c r="B36">
+        <f t="shared" ref="B36" si="22">A36</f>
+        <v>0.96899224806201545</v>
+      </c>
+      <c r="C36" s="14">
+        <v>17</v>
+      </c>
+      <c r="D36" s="1">
+        <f t="shared" si="1"/>
+        <v>8</v>
+      </c>
+      <c r="FK36">
+        <v>0.34087555336940484</v>
+      </c>
+    </row>
+    <row r="37" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <f t="shared" ref="A37" si="23">A36</f>
+        <v>0.96899224806201545</v>
+      </c>
+      <c r="B37">
+        <f>A36*alpha/(1+A36*(alpha-1))</f>
+        <v>0.99364069952305245</v>
+      </c>
+      <c r="C37" s="14"/>
+      <c r="D37" s="1"/>
+      <c r="FK37">
+        <v>0.35103244837758119</v>
+      </c>
+    </row>
+    <row r="38" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <f t="shared" ref="A38" si="24">B37</f>
+        <v>0.99364069952305245</v>
+      </c>
+      <c r="B38">
+        <f t="shared" ref="B38" si="25">A38</f>
+        <v>0.99364069952305245</v>
+      </c>
+      <c r="C38" s="14">
+        <v>18</v>
+      </c>
+      <c r="D38" s="1">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+      <c r="FK38">
+        <v>0.36117936117936117</v>
+      </c>
+    </row>
+    <row r="39" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <f>X_bottom</f>
+        <v>0.2</v>
+      </c>
+      <c r="B39">
+        <f>A39</f>
+        <v>0.2</v>
+      </c>
+      <c r="C39" s="14"/>
+      <c r="D39" s="1"/>
+      <c r="FK39">
+        <v>0.37131630648330061</v>
+      </c>
+    </row>
+    <row r="40" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <f>A39</f>
+        <v>0.2</v>
+      </c>
+      <c r="B40">
+        <f>A39*alpha/(1+A39*(alpha-1))</f>
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="C40" s="14">
+        <v>19</v>
+      </c>
+      <c r="D40" s="1">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="FK40">
+        <v>0.3814432989690722</v>
+      </c>
+    </row>
+    <row r="41" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <f>B40</f>
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="B41">
+        <f>A41</f>
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="C41" s="14"/>
+      <c r="D41" s="1"/>
+      <c r="FK41">
+        <v>0.3915603532875368</v>
+      </c>
+    </row>
+    <row r="42" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <f>A41</f>
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="B42">
+        <f>A42*alpha/(1+A42*(alpha-1))</f>
+        <v>0.86206896551724133</v>
+      </c>
+      <c r="C42" s="14">
+        <v>20</v>
+      </c>
+      <c r="D42" s="1">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="FK42">
+        <v>0.40166748406081415</v>
+      </c>
+    </row>
+    <row r="43" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <f>A42</f>
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="B43">
+        <f>A42*alpha/(1+A42*(alpha-1))</f>
+        <v>0.86206896551724133</v>
+      </c>
+      <c r="C43" s="14"/>
+      <c r="D43" s="1"/>
+      <c r="FK43">
+        <v>0.41176470588235298</v>
+      </c>
+    </row>
+    <row r="44" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <f>X_bottom</f>
+        <v>0.2</v>
+      </c>
+      <c r="B44">
+        <f>A44</f>
+        <v>0.2</v>
+      </c>
+      <c r="C44">
+        <v>21</v>
+      </c>
+      <c r="D44" s="1">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="FK44">
+        <v>0.4218520333170015</v>
+      </c>
+    </row>
+    <row r="45" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A45">
+        <f>A44</f>
+        <v>0.2</v>
+      </c>
+      <c r="B45">
+        <f>A44*alpha/(1+A44*(alpha-1))</f>
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="D45" s="1"/>
+      <c r="FK45">
+        <v>0.43192948090107741</v>
+      </c>
+    </row>
+    <row r="46" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A46">
+        <f>B45</f>
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="B46">
+        <f>A46</f>
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="C46">
+        <v>22</v>
+      </c>
+      <c r="D46" s="1">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="FK46">
+        <v>0.44199706314243759</v>
+      </c>
+    </row>
+    <row r="47" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A47">
+        <f>A46</f>
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="B47">
+        <f>A47*alpha/(1+A47*(alpha-1))</f>
+        <v>0.86206896551724133</v>
+      </c>
+      <c r="D47" s="1"/>
+      <c r="FK47">
+        <v>0.45205479452054798</v>
+      </c>
+    </row>
+    <row r="48" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A48">
+        <f>A47</f>
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="B48">
+        <f>A47*alpha/(1+A47*(alpha-1))</f>
+        <v>0.86206896551724133</v>
+      </c>
+      <c r="C48">
         <v>23</v>
       </c>
-      <c r="FJ26">
-        <v>0.23875432525951557</v>
-      </c>
-    </row>
-    <row r="27" spans="1:166" x14ac:dyDescent="0.3">
-      <c r="A27">
+      <c r="D48" s="1">
         <f t="shared" si="1"/>
-        <v>0.98775589032830391</v>
-      </c>
-      <c r="B27">
-        <f t="shared" si="10"/>
-        <v>0.98775589032830391</v>
-      </c>
-      <c r="C27">
+        <v>2</v>
+      </c>
+      <c r="FK48">
+        <v>0.46210268948655259</v>
+      </c>
+    </row>
+    <row r="49" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A49">
+        <f>B48</f>
+        <v>0.86206896551724133</v>
+      </c>
+      <c r="B49">
+        <f>A49</f>
+        <v>0.86206896551724133</v>
+      </c>
+      <c r="D49" s="1"/>
+      <c r="FK49">
+        <v>0.47214076246334308</v>
+      </c>
+    </row>
+    <row r="50" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <f>A49</f>
+        <v>0.86206896551724133</v>
+      </c>
+      <c r="B50">
+        <f>A49*alpha/(1+A49*(alpha-1))</f>
+        <v>0.96899224806201545</v>
+      </c>
+      <c r="C50">
         <v>24</v>
       </c>
-      <c r="FJ27">
-        <v>0.24901185770750989</v>
-      </c>
-    </row>
-    <row r="28" spans="1:166" x14ac:dyDescent="0.3">
-      <c r="FJ28">
-        <v>0.2592592592592593</v>
-      </c>
-    </row>
-    <row r="29" spans="1:166" x14ac:dyDescent="0.3">
-      <c r="FJ29">
-        <v>0.26949654491609087</v>
-      </c>
-    </row>
-    <row r="30" spans="1:166" x14ac:dyDescent="0.3">
-      <c r="FJ30">
-        <v>0.27972372964972869</v>
-      </c>
-    </row>
-    <row r="31" spans="1:166" x14ac:dyDescent="0.3">
-      <c r="FJ31">
-        <v>0.2899408284023669</v>
-      </c>
-    </row>
-    <row r="32" spans="1:166" x14ac:dyDescent="0.3">
-      <c r="FJ32">
-        <v>0.30014785608674227</v>
-      </c>
-    </row>
-    <row r="33" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ33">
-        <v>0.31034482758620685</v>
-      </c>
-    </row>
-    <row r="34" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ34">
-        <v>0.32053175775480058</v>
-      </c>
-    </row>
-    <row r="35" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ35">
-        <v>0.33070866141732286</v>
-      </c>
-    </row>
-    <row r="36" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ36">
-        <v>0.34087555336940484</v>
-      </c>
-    </row>
-    <row r="37" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ37">
-        <v>0.35103244837758119</v>
-      </c>
-    </row>
-    <row r="38" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ38">
-        <v>0.36117936117936117</v>
-      </c>
-    </row>
-    <row r="39" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ39">
-        <v>0.37131630648330061</v>
-      </c>
-    </row>
-    <row r="40" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ40">
-        <v>0.3814432989690722</v>
-      </c>
-    </row>
-    <row r="41" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ41">
-        <v>0.3915603532875368</v>
-      </c>
-    </row>
-    <row r="42" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ42">
-        <v>0.40166748406081415</v>
-      </c>
-    </row>
-    <row r="43" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ43">
-        <v>0.41176470588235298</v>
-      </c>
-    </row>
-    <row r="44" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ44">
-        <v>0.4218520333170015</v>
-      </c>
-    </row>
-    <row r="45" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ45">
-        <v>0.43192948090107741</v>
-      </c>
-    </row>
-    <row r="46" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ46">
-        <v>0.44199706314243759</v>
-      </c>
-    </row>
-    <row r="47" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ47">
-        <v>0.45205479452054798</v>
-      </c>
-    </row>
-    <row r="48" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ48">
-        <v>0.46210268948655259</v>
-      </c>
-    </row>
-    <row r="49" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ49">
-        <v>0.47214076246334308</v>
-      </c>
-    </row>
-    <row r="50" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ50">
+      <c r="D50" s="1">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="FK50">
         <v>0.48216902784562771</v>
       </c>
     </row>
-    <row r="51" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ51">
+    <row r="51" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="FK51">
         <v>0.4921875</v>
       </c>
     </row>
-    <row r="52" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ52">
+    <row r="52" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="FK52">
         <v>0.50219619326500731</v>
       </c>
     </row>
-    <row r="53" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ53">
+    <row r="53" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="FK53">
         <v>0.51219512195121952</v>
       </c>
     </row>
-    <row r="54" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ54">
+    <row r="54" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="FK54">
         <v>0.52218430034129693</v>
       </c>
     </row>
-    <row r="55" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ55">
+    <row r="55" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="FK55">
         <v>0.53216374269005851</v>
       </c>
     </row>
-    <row r="56" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ56">
+    <row r="56" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="FK56">
         <v>0.54213346322454958</v>
       </c>
     </row>
-    <row r="57" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ57">
+    <row r="57" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="FK57">
         <v>0.55209347614410909</v>
       </c>
     </row>
-    <row r="58" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ58">
+    <row r="58" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="FK58">
         <v>0.56204379562043805</v>
       </c>
     </row>
-    <row r="59" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ59">
+    <row r="59" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="FK59">
         <v>0.57198443579766545</v>
       </c>
     </row>
-    <row r="60" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ60">
+    <row r="60" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="FK60">
         <v>0.58191541079241604</v>
       </c>
     </row>
-    <row r="61" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ61">
+    <row r="61" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="FK61">
         <v>0.59183673469387754</v>
       </c>
     </row>
-    <row r="62" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ62">
+    <row r="62" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="FK62">
         <v>0.60174842156386588</v>
       </c>
     </row>
-    <row r="63" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ63">
+    <row r="63" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="FK63">
         <v>0.61165048543689315</v>
       </c>
     </row>
-    <row r="64" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ64">
+    <row r="64" spans="1:167" x14ac:dyDescent="0.3">
+      <c r="FK64">
         <v>0.62154294032023283</v>
       </c>
     </row>
-    <row r="65" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ65">
+    <row r="65" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK65">
         <v>0.63142580019398631</v>
       </c>
     </row>
-    <row r="66" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ66">
+    <row r="66" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK66">
         <v>0.6412990790111488</v>
       </c>
     </row>
-    <row r="67" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ67">
+    <row r="67" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK67">
         <v>0.65116279069767447</v>
       </c>
     </row>
-    <row r="68" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ68">
+    <row r="68" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK68">
         <v>0.6610169491525425</v>
       </c>
     </row>
-    <row r="69" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ69">
+    <row r="69" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK69">
         <v>0.67086156824782195</v>
       </c>
     </row>
-    <row r="70" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ70">
+    <row r="70" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK70">
         <v>0.68069666182873734</v>
       </c>
     </row>
-    <row r="71" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ71">
+    <row r="71" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK71">
         <v>0.69052224371373316</v>
       </c>
     </row>
-    <row r="72" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ72">
+    <row r="72" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK72">
         <v>0.70033832769453841</v>
       </c>
     </row>
-    <row r="73" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ73">
+    <row r="73" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK73">
         <v>0.71014492753623182</v>
       </c>
     </row>
-    <row r="74" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ74">
+    <row r="74" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK74">
         <v>0.71994205697730551</v>
       </c>
     </row>
-    <row r="75" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ75">
+    <row r="75" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK75">
         <v>0.72972972972972971</v>
       </c>
     </row>
-    <row r="76" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ76">
+    <row r="76" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK76">
         <v>0.73950795947901593</v>
       </c>
     </row>
-    <row r="77" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ77">
+    <row r="77" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK77">
         <v>0.74927675988428166</v>
       </c>
     </row>
-    <row r="78" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ78">
+    <row r="78" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK78">
         <v>0.75903614457831325</v>
       </c>
     </row>
-    <row r="79" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ79">
+    <row r="79" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK79">
         <v>0.76878612716763006</v>
       </c>
     </row>
-    <row r="80" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ80">
+    <row r="80" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK80">
         <v>0.77852672123254707</v>
       </c>
     </row>
-    <row r="81" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ81">
+    <row r="81" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK81">
         <v>0.78825794032723773</v>
       </c>
     </row>
-    <row r="82" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ82">
+    <row r="82" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK82">
         <v>0.79797979797979801</v>
       </c>
     </row>
-    <row r="83" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ83">
+    <row r="83" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK83">
         <v>0.80769230769230771</v>
       </c>
     </row>
-    <row r="84" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ84">
+    <row r="84" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK84">
         <v>0.81739548294089392</v>
       </c>
     </row>
-    <row r="85" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ85">
+    <row r="85" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK85">
         <v>0.82708933717579258</v>
       </c>
     </row>
-    <row r="86" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ86">
+    <row r="86" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK86">
         <v>0.83677388382141127</v>
       </c>
     </row>
-    <row r="87" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ87">
+    <row r="87" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK87">
         <v>0.84644913627639151</v>
       </c>
     </row>
-    <row r="88" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ88">
+    <row r="88" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK88">
         <v>0.85611510791366907</v>
       </c>
     </row>
-    <row r="89" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ89">
+    <row r="89" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK89">
         <v>0.86577181208053677</v>
       </c>
     </row>
-    <row r="90" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ90">
+    <row r="90" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK90">
         <v>0.87541926209870613</v>
       </c>
     </row>
-    <row r="91" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ91">
+    <row r="91" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK91">
         <v>0.88505747126436785</v>
       </c>
     </row>
-    <row r="92" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ92">
+    <row r="92" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK92">
         <v>0.89468645284825288</v>
       </c>
     </row>
-    <row r="93" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ93">
+    <row r="93" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK93">
         <v>0.90430622009569395</v>
       </c>
     </row>
-    <row r="94" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ94">
+    <row r="94" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK94">
         <v>0.91391678622668582</v>
       </c>
     </row>
-    <row r="95" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ95">
+    <row r="95" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK95">
         <v>0.92351816443594648</v>
       </c>
     </row>
-    <row r="96" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ96">
+    <row r="96" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK96">
         <v>0.93311036789297674</v>
       </c>
     </row>
-    <row r="97" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ97">
+    <row r="97" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK97">
         <v>0.94269340974212024</v>
       </c>
     </row>
-    <row r="98" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ98">
+    <row r="98" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK98">
         <v>0.9522673031026252</v>
       </c>
     </row>
-    <row r="99" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ99">
+    <row r="99" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK99">
         <v>0.96183206106870223</v>
       </c>
     </row>
-    <row r="100" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ100">
+    <row r="100" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK100">
         <v>0.97138769670958514</v>
       </c>
     </row>
-    <row r="101" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ101">
+    <row r="101" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK101">
         <v>0.98093422306959011</v>
       </c>
     </row>
-    <row r="102" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ102">
+    <row r="102" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK102">
         <v>0.99047165316817531</v>
       </c>
     </row>
-    <row r="103" spans="166:166" x14ac:dyDescent="0.3">
-      <c r="FJ103">
+    <row r="103" spans="167:167" x14ac:dyDescent="0.3">
+      <c r="FK103">
         <v>1</v>
       </c>
     </row>

</xml_diff>